<commit_message>
Incidentes: consolidado al 26-10 18:12 (ítem 55 con sus 2 medidas cerradas; ítem 32 'Falta turno B'; ítem 84 verificación 'Pendiente Turno B') (xlsx-v18, v=66)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Consolidado Incidentes y Medidas Correctivas (Formato Interno).xlsx
+++ b/Consolidado Incidentes y Medidas Correctivas (Formato Interno).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Entrega de turno 09.04.2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F8D4187-88E1-4B9B-8F2C-07618ACD9B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F54D5589-6F21-4ADD-85CF-8B5124A2B070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -138,7 +138,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1491" uniqueCount="660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1492" uniqueCount="661">
   <si>
     <t xml:space="preserve">INCIDENTES CONTRATO </t>
   </si>
@@ -854,9 +854,6 @@
     <t xml:space="preserve">Difundir informe técnico donde se han identificado los posibles escenarios que puedan ocurrir este tipo de eventos </t>
   </si>
   <si>
-    <t>ABIERTO</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reforzamiento sobre la comunicación en caso de eventos, a quienes de debe dar aviso y acción a seguir posterior a un evento que involucre a equipos. </t>
   </si>
   <si>
@@ -921,6 +918,9 @@
 Supte. General de faena SKIC 
 Cristian Ramirez 
 Codelco</t>
+  </si>
+  <si>
+    <t>ABIERTO</t>
   </si>
   <si>
     <t>Se realizara la actualización del Procedimiento de Perforación manual 4600029025-000000-PROCI-00004 e IPER en donde se incluirán las medidas de control para la exposición a caída de rocas y/o material suelto</t>
@@ -1959,6 +1959,9 @@
 Gerente de construcción
 Hernán Cortes – Mauricio González
 Jefe Deysu.</t>
+  </si>
+  <si>
+    <t>Pendiente Turno B</t>
   </si>
   <si>
     <t>SEGREGACIÓN MANIPULADOR TELESCÓPICO</t>
@@ -7557,8 +7560,8 @@
       <c r="I109" s="35">
         <v>45930</v>
       </c>
-      <c r="J109" s="76" t="s">
-        <v>222</v>
+      <c r="J109" s="78" t="s">
+        <v>218</v>
       </c>
       <c r="K109" s="232"/>
       <c r="L109" s="367"/>
@@ -7572,7 +7575,7 @@
       <c r="E110" s="221"/>
       <c r="F110" s="274"/>
       <c r="G110" s="31" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H110" s="34" t="s">
         <v>220</v>
@@ -7580,8 +7583,8 @@
       <c r="I110" s="35">
         <v>45915</v>
       </c>
-      <c r="J110" s="76" t="s">
-        <v>222</v>
+      <c r="J110" s="78" t="s">
+        <v>218</v>
       </c>
       <c r="K110" s="232"/>
       <c r="L110" s="367"/>
@@ -7598,19 +7601,19 @@
         <v>125</v>
       </c>
       <c r="D111" s="275" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E111" s="226" t="s">
         <v>182</v>
       </c>
       <c r="F111" s="254" t="s">
+        <v>224</v>
+      </c>
+      <c r="G111" s="31" t="s">
         <v>225</v>
       </c>
-      <c r="G111" s="31" t="s">
+      <c r="H111" s="32" t="s">
         <v>226</v>
-      </c>
-      <c r="H111" s="32" t="s">
-        <v>227</v>
       </c>
       <c r="I111" s="35">
         <v>45960</v>
@@ -7636,10 +7639,10 @@
       <c r="E112" s="221"/>
       <c r="F112" s="254"/>
       <c r="G112" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="H112" s="34" t="s">
         <v>228</v>
-      </c>
-      <c r="H112" s="34" t="s">
-        <v>229</v>
       </c>
       <c r="I112" s="35">
         <v>45960</v>
@@ -7659,10 +7662,10 @@
       <c r="E113" s="221"/>
       <c r="F113" s="254"/>
       <c r="G113" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="H113" s="34" t="s">
         <v>230</v>
-      </c>
-      <c r="H113" s="34" t="s">
-        <v>231</v>
       </c>
       <c r="I113" s="35">
         <v>45951</v>
@@ -7682,10 +7685,10 @@
       <c r="E114" s="221"/>
       <c r="F114" s="254"/>
       <c r="G114" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="H114" s="34" t="s">
         <v>232</v>
-      </c>
-      <c r="H114" s="34" t="s">
-        <v>233</v>
       </c>
       <c r="I114" s="35">
         <v>45960</v>
@@ -7705,10 +7708,10 @@
       <c r="E115" s="221"/>
       <c r="F115" s="254"/>
       <c r="G115" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="H115" s="34" t="s">
         <v>234</v>
-      </c>
-      <c r="H115" s="34" t="s">
-        <v>235</v>
       </c>
       <c r="I115" s="35">
         <v>45960</v>
@@ -7731,19 +7734,19 @@
         <v>32</v>
       </c>
       <c r="D116" s="276" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E116" s="206" t="s">
         <v>78</v>
       </c>
       <c r="F116" s="254" t="s">
+        <v>236</v>
+      </c>
+      <c r="G116" s="36" t="s">
         <v>237</v>
       </c>
-      <c r="G116" s="36" t="s">
+      <c r="H116" s="34" t="s">
         <v>238</v>
-      </c>
-      <c r="H116" s="34" t="s">
-        <v>239</v>
       </c>
       <c r="I116" s="35">
         <v>45909</v>
@@ -7752,7 +7755,7 @@
         <v>20</v>
       </c>
       <c r="K116" s="251" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L116" s="265"/>
       <c r="M116" s="12"/>
@@ -7765,16 +7768,16 @@
       <c r="E117" s="207"/>
       <c r="F117" s="254"/>
       <c r="G117" s="36" t="s">
+        <v>240</v>
+      </c>
+      <c r="H117" s="34" t="s">
         <v>241</v>
-      </c>
-      <c r="H117" s="34" t="s">
-        <v>242</v>
       </c>
       <c r="I117" s="35">
         <v>45930</v>
       </c>
       <c r="J117" s="76" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K117" s="251"/>
       <c r="L117" s="265"/>
@@ -7791,7 +7794,7 @@
         <v>243</v>
       </c>
       <c r="H118" s="34" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I118" s="35">
         <v>45930</v>
@@ -7820,7 +7823,7 @@
         <v>45930</v>
       </c>
       <c r="J119" s="76" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K119" s="251"/>
       <c r="L119" s="265"/>
@@ -7843,7 +7846,7 @@
         <v>45930</v>
       </c>
       <c r="J120" s="76" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K120" s="251"/>
       <c r="L120" s="265"/>
@@ -7879,7 +7882,7 @@
         <v>20</v>
       </c>
       <c r="K121" s="240" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L121" s="221"/>
       <c r="M121" s="12"/>
@@ -7983,7 +7986,7 @@
         <v>20</v>
       </c>
       <c r="K125" s="240" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L125" s="221" t="s">
         <v>22</v>
@@ -8157,7 +8160,7 @@
         <v>20</v>
       </c>
       <c r="K131" s="251" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L131" s="221" t="s">
         <v>22</v>
@@ -8273,7 +8276,7 @@
         <v>20</v>
       </c>
       <c r="K135" s="251" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L135" s="221"/>
       <c r="M135" s="12"/>
@@ -8356,7 +8359,7 @@
         <v>20</v>
       </c>
       <c r="K138" s="240" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="L138" s="221" t="s">
         <v>22</v>
@@ -8431,7 +8434,7 @@
         <v>287</v>
       </c>
       <c r="H142" s="32" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I142" s="6">
         <v>45996</v>
@@ -8456,7 +8459,7 @@
         <v>288</v>
       </c>
       <c r="H143" s="32" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I143" s="6">
         <v>45996</v>
@@ -9290,7 +9293,7 @@
         <v>125</v>
       </c>
       <c r="D175" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E175" s="89" t="s">
         <v>182</v>
@@ -9302,7 +9305,7 @@
         <v>350</v>
       </c>
       <c r="H175" s="32" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I175" s="4">
         <v>46061</v>
@@ -9349,7 +9352,7 @@
         <v>46380</v>
       </c>
       <c r="J176" s="50" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K176" s="239" t="s">
         <v>22</v>
@@ -9432,7 +9435,7 @@
         <v>46079</v>
       </c>
       <c r="J179" s="50" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K179" s="239" t="s">
         <v>22</v>
@@ -9600,7 +9603,7 @@
         <v>46081</v>
       </c>
       <c r="J185" s="69" t="s">
-        <v>222</v>
+        <v>20</v>
       </c>
       <c r="K185" s="98" t="s">
         <v>22</v>
@@ -9623,7 +9626,7 @@
         <v>46140</v>
       </c>
       <c r="J186" s="69" t="s">
-        <v>222</v>
+        <v>20</v>
       </c>
       <c r="K186" s="98" t="s">
         <v>22</v>
@@ -9739,7 +9742,7 @@
         <v>46069</v>
       </c>
       <c r="J190" s="82" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K190" s="232" t="s">
         <v>22</v>
@@ -9824,7 +9827,7 @@
         <v>46082</v>
       </c>
       <c r="J193" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K193" s="232"/>
       <c r="L193" s="221"/>
@@ -9882,7 +9885,7 @@
         <v>46111</v>
       </c>
       <c r="J195" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K195" s="85" t="s">
         <v>22</v>
@@ -9942,7 +9945,7 @@
         <v>46111</v>
       </c>
       <c r="J197" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K197" s="85"/>
       <c r="L197" s="12"/>
@@ -9963,7 +9966,7 @@
         <v>46111</v>
       </c>
       <c r="J198" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K198" s="85"/>
       <c r="L198" s="12"/>
@@ -10017,7 +10020,7 @@
         <v>46080</v>
       </c>
       <c r="J200" s="83" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K200" s="95"/>
       <c r="L200" s="12"/>
@@ -10085,7 +10088,7 @@
         <v>46147</v>
       </c>
       <c r="J202" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K202" s="107"/>
       <c r="L202" s="5"/>
@@ -17441,7 +17444,7 @@
         <v>420</v>
       </c>
       <c r="J205" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K205" s="107"/>
       <c r="L205" s="5"/>
@@ -22349,7 +22352,7 @@
         <v>420</v>
       </c>
       <c r="J207" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K207" s="107"/>
       <c r="L207" s="5"/>
@@ -24809,7 +24812,7 @@
         <v>46142</v>
       </c>
       <c r="J208" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K208" s="107"/>
       <c r="L208" s="5"/>
@@ -32153,7 +32156,7 @@
         <v>46143</v>
       </c>
       <c r="J211" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K211" s="108"/>
       <c r="L211" s="2"/>
@@ -34613,7 +34616,7 @@
         <v>46142</v>
       </c>
       <c r="J212" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K212" s="108" t="s">
         <v>440</v>
@@ -44421,7 +44424,7 @@
         <v>447</v>
       </c>
       <c r="J216" s="87" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K216" s="108"/>
       <c r="L216" s="2"/>
@@ -54237,7 +54240,7 @@
         <v>46137</v>
       </c>
       <c r="J220" s="87" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K220" s="108"/>
       <c r="L220" s="2"/>
@@ -56685,7 +56688,7 @@
         <v>46137</v>
       </c>
       <c r="J221" s="92" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K221" s="90"/>
       <c r="L221" s="2"/>
@@ -59207,7 +59210,7 @@
         <v>469</v>
       </c>
       <c r="J224" s="83" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K224" s="95"/>
       <c r="L224" s="12"/>
@@ -59323,7 +59326,7 @@
         <v>46142</v>
       </c>
       <c r="J228" s="69" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K228" s="110"/>
       <c r="L228" s="12"/>
@@ -59427,7 +59430,7 @@
         <v>46141</v>
       </c>
       <c r="J232" s="5" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K232" s="110" t="s">
         <v>22</v>
@@ -59510,7 +59513,7 @@
         <v>498</v>
       </c>
       <c r="J235" s="5" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K235" s="128"/>
       <c r="L235" s="60"/>
@@ -59533,7 +59536,7 @@
         <v>498</v>
       </c>
       <c r="J236" s="5" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K236" s="85"/>
       <c r="L236" s="56"/>
@@ -59595,7 +59598,7 @@
         <v>46172</v>
       </c>
       <c r="J238" s="98" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K238" s="5"/>
       <c r="L238" s="98"/>
@@ -59757,7 +59760,7 @@
       <c r="H244" s="60"/>
       <c r="I244" s="142"/>
       <c r="J244" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K244" s="60"/>
       <c r="L244" s="60"/>
@@ -59776,7 +59779,7 @@
       <c r="H245" s="5"/>
       <c r="I245" s="4"/>
       <c r="J245" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K245" s="5"/>
       <c r="L245" s="5"/>
@@ -59807,7 +59810,7 @@
       <c r="H246" s="5"/>
       <c r="I246" s="4"/>
       <c r="J246" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K246" s="5"/>
       <c r="L246" s="5"/>
@@ -59923,9 +59926,11 @@
         <v>46164</v>
       </c>
       <c r="J250" s="129" t="s">
-        <v>222</v>
-      </c>
-      <c r="K250" s="5"/>
+        <v>242</v>
+      </c>
+      <c r="K250" s="5" t="s">
+        <v>543</v>
+      </c>
       <c r="L250" s="5"/>
       <c r="M250" s="5"/>
     </row>
@@ -59940,25 +59945,25 @@
         <v>501</v>
       </c>
       <c r="D251" s="206" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E251" s="200" t="s">
         <v>521</v>
       </c>
       <c r="F251" s="214" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="G251" s="14" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="H251" s="144" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="I251" s="4">
         <v>46188</v>
       </c>
       <c r="J251" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K251" s="5"/>
       <c r="L251" s="5"/>
@@ -59972,16 +59977,16 @@
       <c r="E252" s="201"/>
       <c r="F252" s="338"/>
       <c r="G252" s="100" t="s">
+        <v>548</v>
+      </c>
+      <c r="H252" s="144" t="s">
         <v>547</v>
-      </c>
-      <c r="H252" s="144" t="s">
-        <v>546</v>
       </c>
       <c r="I252" s="4">
         <v>46188</v>
       </c>
       <c r="J252" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K252" s="5"/>
       <c r="L252" s="5"/>
@@ -59995,10 +60000,10 @@
       <c r="E253" s="201"/>
       <c r="F253" s="338"/>
       <c r="G253" s="100" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="H253" s="144" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="I253" s="4">
         <v>46188</v>
@@ -60018,16 +60023,16 @@
       <c r="E254" s="201"/>
       <c r="F254" s="338"/>
       <c r="G254" s="100" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="H254" s="144" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="I254" s="4">
         <v>46188</v>
       </c>
       <c r="J254" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K254" s="5"/>
       <c r="L254" s="5"/>
@@ -60041,16 +60046,16 @@
       <c r="E255" s="201"/>
       <c r="F255" s="338"/>
       <c r="G255" s="100" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="H255" s="144" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="I255" s="4">
         <v>46188</v>
       </c>
       <c r="J255" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K255" s="5"/>
       <c r="L255" s="5"/>
@@ -60067,25 +60072,25 @@
         <v>265</v>
       </c>
       <c r="D256" s="220" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="E256" s="221" t="s">
         <v>521</v>
       </c>
       <c r="F256" s="339" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="G256" s="163" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="H256" s="144" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="I256" s="143">
         <v>46203</v>
       </c>
       <c r="J256" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K256" s="138"/>
       <c r="L256" s="5"/>
@@ -60099,16 +60104,16 @@
       <c r="E257" s="221"/>
       <c r="F257" s="227"/>
       <c r="G257" s="163" t="s">
+        <v>558</v>
+      </c>
+      <c r="H257" s="144" t="s">
         <v>557</v>
-      </c>
-      <c r="H257" s="144" t="s">
-        <v>556</v>
       </c>
       <c r="I257" s="143">
         <v>46203</v>
       </c>
       <c r="J257" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K257" s="138"/>
       <c r="L257" s="5"/>
@@ -60122,7 +60127,7 @@
       <c r="E258" s="221"/>
       <c r="F258" s="227"/>
       <c r="G258" s="163" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="H258" s="144" t="s">
         <v>540</v>
@@ -60131,7 +60136,7 @@
         <v>46203</v>
       </c>
       <c r="J258" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K258" s="138"/>
       <c r="L258" s="5"/>
@@ -60145,7 +60150,7 @@
       <c r="E259" s="200"/>
       <c r="F259" s="228"/>
       <c r="G259" s="164" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="H259" s="58" t="s">
         <v>540</v>
@@ -60171,19 +60176,19 @@
         <v>32</v>
       </c>
       <c r="D260" s="220" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E260" s="221" t="s">
         <v>27</v>
       </c>
       <c r="F260" s="337" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="G260" s="13" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="H260" s="2" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="I260" s="4"/>
       <c r="J260" s="5"/>
@@ -60199,14 +60204,14 @@
       <c r="E261" s="221"/>
       <c r="F261" s="220"/>
       <c r="G261" s="13" t="s">
+        <v>565</v>
+      </c>
+      <c r="H261" s="2" t="s">
         <v>564</v>
-      </c>
-      <c r="H261" s="2" t="s">
-        <v>563</v>
       </c>
       <c r="I261" s="5"/>
       <c r="J261" s="5" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K261" s="5"/>
       <c r="L261" s="5"/>
@@ -60223,25 +60228,25 @@
         <v>32</v>
       </c>
       <c r="D262" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E262" s="2" t="s">
         <v>521</v>
       </c>
       <c r="F262" s="13" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="G262" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="H262" s="2" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="I262" s="4">
         <v>46193</v>
       </c>
       <c r="J262" s="5" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K262" s="5"/>
       <c r="L262" s="5"/>
@@ -60258,16 +60263,16 @@
         <v>501</v>
       </c>
       <c r="D263" s="58" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="E263" s="56" t="s">
         <v>27</v>
       </c>
       <c r="F263" s="137" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="G263" s="56" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="H263" s="56"/>
       <c r="I263" s="56"/>
@@ -60277,7 +60282,7 @@
       <c r="K263" s="5"/>
       <c r="L263" s="5"/>
       <c r="M263" s="58" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="264" spans="1:13" ht="81" customHeight="1">
@@ -60291,22 +60296,22 @@
         <v>125</v>
       </c>
       <c r="D264" s="206" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="E264" s="200" t="s">
         <v>521</v>
       </c>
       <c r="F264" s="214" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="G264" s="56" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="H264" s="56" t="s">
         <v>358</v>
       </c>
       <c r="I264" s="56" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="J264" s="93" t="s">
         <v>20</v>
@@ -60323,16 +60328,16 @@
       <c r="E265" s="201"/>
       <c r="F265" s="338"/>
       <c r="G265" s="56" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="H265" s="56" t="s">
         <v>358</v>
       </c>
       <c r="I265" s="56" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="J265" s="93" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K265" s="56"/>
       <c r="L265" s="85"/>
@@ -60346,13 +60351,13 @@
       <c r="E266" s="202"/>
       <c r="F266" s="215"/>
       <c r="G266" s="56" t="s">
+        <v>579</v>
+      </c>
+      <c r="H266" s="56" t="s">
+        <v>580</v>
+      </c>
+      <c r="I266" s="56" t="s">
         <v>578</v>
-      </c>
-      <c r="H266" s="56" t="s">
-        <v>579</v>
-      </c>
-      <c r="I266" s="56" t="s">
-        <v>577</v>
       </c>
       <c r="J266" s="93" t="s">
         <v>20</v>
@@ -60369,33 +60374,33 @@
         <v>46201</v>
       </c>
       <c r="C267" s="220" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="D267" s="220" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E267" s="226" t="s">
         <v>199</v>
       </c>
       <c r="F267" s="346" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="G267" s="150" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="H267" s="2" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="I267" s="4">
         <v>46223</v>
       </c>
       <c r="J267" s="129" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K267" s="111"/>
       <c r="L267" s="12"/>
       <c r="M267" s="345" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="268" spans="1:13" ht="44.25" customHeight="1">
@@ -60406,16 +60411,16 @@
       <c r="E268" s="226"/>
       <c r="F268" s="346"/>
       <c r="G268" s="14" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="H268" s="2" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="I268" s="4">
         <v>46223</v>
       </c>
       <c r="J268" s="138" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K268" s="169"/>
       <c r="L268" s="170"/>
@@ -60429,10 +60434,10 @@
       <c r="E269" s="347"/>
       <c r="F269" s="216"/>
       <c r="G269" s="139" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="H269" s="58" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="I269" s="57">
         <v>46223</v>
@@ -60455,25 +60460,25 @@
         <v>501</v>
       </c>
       <c r="D270" s="356" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="E270" s="355" t="s">
         <v>27</v>
       </c>
       <c r="F270" s="353" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="G270" s="166" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="H270" s="58" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="I270" s="57">
         <v>46233</v>
       </c>
       <c r="J270" s="56" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K270" s="56"/>
       <c r="L270" s="56"/>
@@ -60487,16 +60492,16 @@
       <c r="E271" s="212"/>
       <c r="F271" s="354"/>
       <c r="G271" s="14" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="H271" s="176" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="I271" s="57">
         <v>46233</v>
       </c>
       <c r="J271" s="56" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K271" s="167"/>
       <c r="L271" s="60"/>
@@ -60513,13 +60518,13 @@
         <v>265</v>
       </c>
       <c r="D272" s="2" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E272" s="5" t="s">
         <v>199</v>
       </c>
       <c r="F272" s="13" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="G272" s="190" t="s">
         <v>30</v>
@@ -60554,19 +60559,19 @@
         <v>265</v>
       </c>
       <c r="D273" s="208" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="E273" s="348" t="s">
         <v>320</v>
       </c>
       <c r="F273" s="218" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="G273" s="13" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="H273" s="189" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="I273" s="4">
         <v>46280</v>
@@ -60577,7 +60582,7 @@
       <c r="K273" s="12"/>
       <c r="L273" s="12"/>
       <c r="M273" s="337" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
     </row>
     <row r="274" spans="1:13" ht="68.25" customHeight="1">
@@ -60588,16 +60593,16 @@
       <c r="E274" s="266"/>
       <c r="F274" s="346"/>
       <c r="G274" s="187" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="H274" s="175" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="I274" s="4">
         <v>46295</v>
       </c>
       <c r="J274" s="5" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K274" s="12"/>
       <c r="L274" s="12"/>
@@ -60611,10 +60616,10 @@
       <c r="E275" s="266"/>
       <c r="F275" s="337"/>
       <c r="G275" s="191" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H275" s="175" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="I275" s="4">
         <v>46265</v>
@@ -60634,10 +60639,10 @@
       <c r="E276" s="266"/>
       <c r="F276" s="346"/>
       <c r="G276" s="13" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="H276" s="175" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="I276" s="4">
         <v>46295</v>
@@ -60657,10 +60662,10 @@
       <c r="E277" s="266"/>
       <c r="F277" s="346"/>
       <c r="G277" s="13" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="H277" s="176" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="I277" s="4">
         <v>46295</v>
@@ -60680,10 +60685,10 @@
       <c r="E278" s="266"/>
       <c r="F278" s="346"/>
       <c r="G278" s="116" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="H278" s="127" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="I278" s="4">
         <v>46295</v>
@@ -60703,16 +60708,16 @@
       <c r="E279" s="266"/>
       <c r="F279" s="346"/>
       <c r="G279" s="187" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="H279" s="175" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="I279" s="4">
         <v>46295</v>
       </c>
       <c r="J279" s="5" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K279" s="12"/>
       <c r="L279" s="12"/>
@@ -60726,16 +60731,16 @@
       <c r="E280" s="349"/>
       <c r="F280" s="216"/>
       <c r="G280" s="181" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="H280" s="175" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="I280" s="4">
         <v>46295</v>
       </c>
       <c r="J280" s="192" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="K280" s="12"/>
       <c r="L280" s="12"/>
@@ -60752,19 +60757,19 @@
         <v>265</v>
       </c>
       <c r="D281" s="206" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E281" s="342" t="s">
         <v>27</v>
       </c>
       <c r="F281" s="216" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="G281" s="188" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="H281" s="168" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="I281" s="179">
         <v>46315</v>
@@ -60783,16 +60788,16 @@
       <c r="E282" s="343"/>
       <c r="F282" s="217"/>
       <c r="G282" s="188" t="s">
+        <v>620</v>
+      </c>
+      <c r="H282" s="168" t="s">
         <v>619</v>
-      </c>
-      <c r="H282" s="168" t="s">
-        <v>618</v>
       </c>
       <c r="I282" s="171">
         <v>46315</v>
       </c>
       <c r="J282" s="5" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K282" s="174"/>
       <c r="L282" s="95"/>
@@ -60806,7 +60811,7 @@
       <c r="E283" s="344"/>
       <c r="F283" s="218"/>
       <c r="G283" s="188" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="H283" s="168" t="s">
         <v>88</v>
@@ -60815,7 +60820,7 @@
         <v>46315</v>
       </c>
       <c r="J283" s="56" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K283" s="174"/>
       <c r="L283" s="95"/>
@@ -60832,19 +60837,19 @@
         <v>265</v>
       </c>
       <c r="D284" s="206" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E284" s="200" t="s">
         <v>182</v>
       </c>
       <c r="F284" s="216" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="G284" s="13" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="H284" s="134" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="I284" s="147">
         <v>46295</v>
@@ -60855,7 +60860,7 @@
       <c r="K284" s="193"/>
       <c r="L284" s="60"/>
       <c r="M284" s="214" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
     </row>
     <row r="285" spans="1:13" ht="96.75" customHeight="1">
@@ -60866,16 +60871,16 @@
       <c r="E285" s="202"/>
       <c r="F285" s="218"/>
       <c r="G285" s="14" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="H285" s="134" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="I285" s="171">
         <v>46295</v>
       </c>
       <c r="J285" s="5" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K285" s="174"/>
       <c r="L285" s="60"/>
@@ -60892,19 +60897,19 @@
         <v>125</v>
       </c>
       <c r="D286" s="220" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E286" s="212" t="s">
         <v>521</v>
       </c>
       <c r="F286" s="216" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="G286" s="13" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="H286" s="93" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="I286" s="171">
         <v>46285</v>
@@ -60924,10 +60929,10 @@
       <c r="E287" s="219"/>
       <c r="F287" s="217"/>
       <c r="G287" s="13" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="H287" s="93" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="I287" s="171">
         <v>46285</v>
@@ -60947,10 +60952,10 @@
       <c r="E288" s="213"/>
       <c r="F288" s="218"/>
       <c r="G288" s="13" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="H288" s="93" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="I288" s="171">
         <v>46285</v>
@@ -60973,13 +60978,13 @@
         <v>125</v>
       </c>
       <c r="D289" s="200" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="E289" s="200" t="s">
         <v>27</v>
       </c>
       <c r="F289" s="206" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="G289" s="12"/>
       <c r="H289" s="167"/>
@@ -60997,10 +61002,10 @@
       <c r="E290" s="201"/>
       <c r="F290" s="207"/>
       <c r="G290" s="194" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="H290" s="195" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="I290" s="95"/>
       <c r="J290" s="12"/>
@@ -61034,28 +61039,28 @@
         <v>125</v>
       </c>
       <c r="D292" s="200" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E292" s="200" t="s">
         <v>182</v>
       </c>
       <c r="F292" s="206" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="G292" s="194" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="H292" s="196" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="I292" s="197">
         <v>46310</v>
       </c>
       <c r="J292" s="177" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K292" s="60" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="L292" s="60"/>
       <c r="M292" s="60"/>
@@ -61068,7 +61073,7 @@
       <c r="E293" s="202"/>
       <c r="F293" s="208"/>
       <c r="G293" s="194" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="H293" s="93" t="s">
         <v>257</v>
@@ -61077,10 +61082,10 @@
         <v>46310</v>
       </c>
       <c r="J293" s="60" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K293" s="60" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="L293" s="60"/>
       <c r="M293" s="60"/>
@@ -61096,25 +61101,25 @@
         <v>265</v>
       </c>
       <c r="D294" s="206" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="E294" s="206" t="s">
         <v>27</v>
       </c>
       <c r="F294" s="206" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="G294" s="139" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="H294" s="194" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="I294" s="197">
         <v>46325</v>
       </c>
       <c r="J294" s="60" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K294" s="60"/>
       <c r="L294" s="60"/>
@@ -61128,16 +61133,16 @@
       <c r="E295" s="207"/>
       <c r="F295" s="207"/>
       <c r="G295" s="139" t="s">
+        <v>651</v>
+      </c>
+      <c r="H295" s="194" t="s">
         <v>650</v>
-      </c>
-      <c r="H295" s="194" t="s">
-        <v>649</v>
       </c>
       <c r="I295" s="197">
         <v>46325</v>
       </c>
       <c r="J295" s="60" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K295" s="60"/>
       <c r="L295" s="60"/>
@@ -61154,25 +61159,25 @@
         <v>125</v>
       </c>
       <c r="D296" s="206" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="E296" s="206" t="s">
         <v>521</v>
       </c>
       <c r="F296" s="206" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="G296" s="198" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="H296" s="194" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="I296" s="197">
         <v>46325</v>
       </c>
       <c r="J296" s="60" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
       <c r="K296" s="12"/>
       <c r="L296" s="12"/>
@@ -61186,16 +61191,16 @@
       <c r="E297" s="207"/>
       <c r="F297" s="207"/>
       <c r="G297" s="114" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="H297" s="194" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="I297" s="197">
         <v>46325</v>
       </c>
       <c r="J297" s="60" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
     </row>
     <row r="298" spans="1:13" ht="39.75" customHeight="1">
@@ -61206,16 +61211,16 @@
       <c r="E298" s="208"/>
       <c r="F298" s="209"/>
       <c r="G298" s="14" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="H298" s="100" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="I298" s="199">
         <v>46325</v>
       </c>
       <c r="J298" s="12" t="s">
-        <v>222</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -61893,7 +61898,7 @@
     <mergeCell ref="E294:E295"/>
     <mergeCell ref="F294:F295"/>
   </mergeCells>
-  <conditionalFormatting sqref="J2:J66 J155:J170 I142:I145 J222 J227 J69:J138 J142:J150 J175:J214 J232:J271 J273:J1048576">
+  <conditionalFormatting sqref="J2:J66 J155:J170 I142:I145 J222 J227 J142:J150 J175:J214 J232:J271 J273:J1048576 J69:J138">
     <cfRule type="cellIs" dxfId="32" priority="36" operator="equal">
       <formula>"ABIERTO"</formula>
     </cfRule>
@@ -61901,7 +61906,7 @@
       <formula>NOT(ISERROR(SEARCH("ABIERTO",I2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J66 J222 J227 J69:J138 J142:J170 J175:J214 J232:J271 J273:J1048576">
+  <conditionalFormatting sqref="J2:J66 J222 J227 J142:J170 J175:J214 J232:J271 J273:J1048576 J69:J138">
     <cfRule type="containsText" dxfId="30" priority="35" operator="containsText" text="ABIERTO">
       <formula>NOT(ISERROR(SEARCH("ABIERTO",J2)))</formula>
     </cfRule>
@@ -62098,13 +62103,13 @@
         <v>501</v>
       </c>
       <c r="E7" s="206" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F7" s="200" t="s">
         <v>521</v>
       </c>
       <c r="G7" s="214" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="8" spans="2:7" hidden="1">
@@ -62150,13 +62155,13 @@
         <v>501</v>
       </c>
       <c r="E12" s="206" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F12" s="200" t="s">
         <v>521</v>
       </c>
       <c r="G12" s="214" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="13" spans="2:7" hidden="1">
@@ -62194,18 +62199,18 @@
         <v>32</v>
       </c>
       <c r="E16" s="58" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="F16" s="56" t="s">
         <v>27</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="76.5" customHeight="1">
       <c r="B17" s="360" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="C17" s="361"/>
       <c r="D17" s="361"/>
@@ -62461,13 +62466,13 @@
         <v>501</v>
       </c>
       <c r="D33" s="58" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E33" s="56" t="s">
         <v>521</v>
       </c>
       <c r="F33" s="137" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="34" spans="2:8" ht="76.5">
@@ -62478,18 +62483,18 @@
         <v>501</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>521</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="36" spans="2:8">
       <c r="B36" s="363" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C36" s="364"/>
       <c r="D36" s="364"/>
@@ -62674,7 +62679,7 @@
         <v>45856</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>172</v>
@@ -62691,7 +62696,7 @@
         <v>45895</v>
       </c>
       <c r="C48" s="21" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D48" s="21" t="s">
         <v>213</v>
@@ -62708,7 +62713,7 @@
         <v>45911</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>247</v>
@@ -62759,7 +62764,7 @@
         <v>45952</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>276</v>
@@ -62847,13 +62852,13 @@
         <v>32</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>27</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
   </sheetData>

</xml_diff>